<commit_message>
Wszystko działa - czyścimy
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/pna/KorektyPna.xlsx
+++ b/TerytLoad/AppData/pna/KorektyPna.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\pna\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9138A7D-7B73-49DB-B019-B5DDC296B200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6467CE16-A1A4-4056-AFAF-3F235DF20CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{09E8D2D0-BB12-495B-A39A-B0FC9433E411}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="941" uniqueCount="257">
   <si>
     <t>13-332</t>
   </si>
@@ -747,6 +747,66 @@
   </si>
   <si>
     <t>park Źródliska I (Palmiarnia)</t>
+  </si>
+  <si>
+    <t>30-698</t>
+  </si>
+  <si>
+    <t>Tuchowska</t>
+  </si>
+  <si>
+    <t>1-DK</t>
+  </si>
+  <si>
+    <t>Kraków</t>
+  </si>
+  <si>
+    <t>małopolskie</t>
+  </si>
+  <si>
+    <t>45-DK(n) 50-DK(p)</t>
+  </si>
+  <si>
+    <t>30-619</t>
+  </si>
+  <si>
+    <t>Turniejowa</t>
+  </si>
+  <si>
+    <t>57-DK</t>
+  </si>
+  <si>
+    <t>Nakładający się zakres</t>
+  </si>
+  <si>
+    <t>57-59(n) 61-DK(n) 24-DK(p)</t>
+  </si>
+  <si>
+    <t>30-418</t>
+  </si>
+  <si>
+    <t>Zakopiańska</t>
+  </si>
+  <si>
+    <t>33-147(n), 46-58b(p), 62-70a(p)</t>
+  </si>
+  <si>
+    <t>33-147(n),46-58b(p),62(p),64-70a(p)</t>
+  </si>
+  <si>
+    <t>30-435</t>
+  </si>
+  <si>
+    <t>60-62b(p), 72-264(p), 149-DK(n), 265-277</t>
+  </si>
+  <si>
+    <t>60,62a-62b(p),72-264(p),149-DK(n),265-277</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kraków </t>
+  </si>
+  <si>
+    <t>Ulica w postaci odwrotnej</t>
   </si>
 </sst>
 </file>
@@ -1119,13 +1179,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79EC6EBE-762D-4FEE-AB4D-0625E60C23B9}">
-  <dimension ref="A1:H177"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32.42578125" customWidth="1"/>
     <col min="3" max="3" width="42.42578125" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="42.85546875" customWidth="1"/>
     <col min="5" max="5" width="22.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
@@ -2712,7 +2772,7 @@
         <v>142</v>
       </c>
       <c r="H88" t="s">
-        <v>103</v>
+        <v>256</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -2869,7 +2929,7 @@
         <v>52</v>
       </c>
       <c r="H96" t="s">
-        <v>106</v>
+        <v>256</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.25">
@@ -3346,7 +3406,7 @@
         <v>59</v>
       </c>
       <c r="H126" t="s">
-        <v>108</v>
+        <v>256</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.25">
@@ -3473,7 +3533,7 @@
         <v>52</v>
       </c>
       <c r="H134" t="s">
-        <v>109</v>
+        <v>256</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.25">
@@ -3740,7 +3800,7 @@
         <v>52</v>
       </c>
       <c r="H152" t="s">
-        <v>110</v>
+        <v>256</v>
       </c>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.25">
@@ -4063,7 +4123,7 @@
         <v>52</v>
       </c>
       <c r="H174" t="s">
-        <v>111</v>
+        <v>256</v>
       </c>
     </row>
     <row r="175" spans="1:8" x14ac:dyDescent="0.25">
@@ -4109,7 +4169,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>234</v>
       </c>
@@ -4127,6 +4187,202 @@
       </c>
       <c r="G177" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>237</v>
+      </c>
+      <c r="B178" t="s">
+        <v>240</v>
+      </c>
+      <c r="C178" t="s">
+        <v>238</v>
+      </c>
+      <c r="D178" t="s">
+        <v>239</v>
+      </c>
+      <c r="E178" t="s">
+        <v>240</v>
+      </c>
+      <c r="F178" t="s">
+        <v>240</v>
+      </c>
+      <c r="G178" t="s">
+        <v>241</v>
+      </c>
+      <c r="H178" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>237</v>
+      </c>
+      <c r="B179" t="s">
+        <v>240</v>
+      </c>
+      <c r="C179" t="s">
+        <v>238</v>
+      </c>
+      <c r="D179" t="s">
+        <v>242</v>
+      </c>
+      <c r="E179" t="s">
+        <v>240</v>
+      </c>
+      <c r="F179" t="s">
+        <v>240</v>
+      </c>
+      <c r="G179" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>243</v>
+      </c>
+      <c r="B180" t="s">
+        <v>240</v>
+      </c>
+      <c r="C180" t="s">
+        <v>244</v>
+      </c>
+      <c r="D180" t="s">
+        <v>245</v>
+      </c>
+      <c r="E180" t="s">
+        <v>240</v>
+      </c>
+      <c r="F180" t="s">
+        <v>240</v>
+      </c>
+      <c r="G180" t="s">
+        <v>241</v>
+      </c>
+      <c r="H180" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>243</v>
+      </c>
+      <c r="B181" t="s">
+        <v>240</v>
+      </c>
+      <c r="C181" t="s">
+        <v>244</v>
+      </c>
+      <c r="D181" t="s">
+        <v>247</v>
+      </c>
+      <c r="E181" t="s">
+        <v>240</v>
+      </c>
+      <c r="F181" t="s">
+        <v>240</v>
+      </c>
+      <c r="G181" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>248</v>
+      </c>
+      <c r="B182" t="s">
+        <v>240</v>
+      </c>
+      <c r="C182" t="s">
+        <v>249</v>
+      </c>
+      <c r="D182" t="s">
+        <v>250</v>
+      </c>
+      <c r="E182" t="s">
+        <v>240</v>
+      </c>
+      <c r="F182" t="s">
+        <v>240</v>
+      </c>
+      <c r="G182" t="s">
+        <v>241</v>
+      </c>
+      <c r="H182" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>248</v>
+      </c>
+      <c r="B183" t="s">
+        <v>240</v>
+      </c>
+      <c r="C183" t="s">
+        <v>249</v>
+      </c>
+      <c r="D183" t="s">
+        <v>251</v>
+      </c>
+      <c r="E183" t="s">
+        <v>240</v>
+      </c>
+      <c r="F183" t="s">
+        <v>240</v>
+      </c>
+      <c r="G183" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>252</v>
+      </c>
+      <c r="B184" t="s">
+        <v>240</v>
+      </c>
+      <c r="C184" t="s">
+        <v>249</v>
+      </c>
+      <c r="D184" t="s">
+        <v>253</v>
+      </c>
+      <c r="E184" t="s">
+        <v>240</v>
+      </c>
+      <c r="F184" t="s">
+        <v>240</v>
+      </c>
+      <c r="G184" t="s">
+        <v>241</v>
+      </c>
+      <c r="H184" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>252</v>
+      </c>
+      <c r="B185" t="s">
+        <v>255</v>
+      </c>
+      <c r="C185" t="s">
+        <v>249</v>
+      </c>
+      <c r="D185" t="s">
+        <v>254</v>
+      </c>
+      <c r="E185" t="s">
+        <v>240</v>
+      </c>
+      <c r="F185" t="s">
+        <v>240</v>
+      </c>
+      <c r="G185" t="s">
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Całe PNA ładuje sie prawidłowo
</commit_message>
<xml_diff>
--- a/TerytLoad/AppData/pna/KorektyPna.xlsx
+++ b/TerytLoad/AppData/pna/KorektyPna.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\src\TerytLoad\TerytLoad\AppData\pna\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4C7654-8187-473C-B4C9-8024AA076269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6570AD58-AC18-4AF3-9DA2-BC4996F9BFE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2797" uniqueCount="557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2781" uniqueCount="556">
   <si>
     <t>Kod</t>
   </si>
@@ -1062,9 +1062,6 @@
   </si>
   <si>
     <t>ONZ Rondo</t>
-  </si>
-  <si>
-    <t>Rondo ONZ</t>
   </si>
   <si>
     <t>89-600</t>
@@ -2582,7 +2579,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I421"/>
+  <dimension ref="A1:I419"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -2604,7 +2601,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
@@ -3672,7 +3669,7 @@
         <v>70</v>
       </c>
       <c r="I46" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -3683,7 +3680,7 @@
         <v>68</v>
       </c>
       <c r="D47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E47" t="s">
         <v>11</v>
@@ -5755,7 +5752,7 @@
         <v>127</v>
       </c>
       <c r="D156" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="E156" t="s">
         <v>11</v>
@@ -6044,7 +6041,7 @@
         <v>17</v>
       </c>
       <c r="I170" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.25">
@@ -6055,7 +6052,7 @@
         <v>127</v>
       </c>
       <c r="D171" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="E171" t="s">
         <v>11</v>
@@ -6133,7 +6130,7 @@
         <v>17</v>
       </c>
       <c r="I174" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
@@ -6144,7 +6141,7 @@
         <v>127</v>
       </c>
       <c r="D175" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="E175" t="s">
         <v>11</v>
@@ -6196,7 +6193,7 @@
         <v>127</v>
       </c>
       <c r="D177" t="s">
-        <v>343</v>
+        <v>367</v>
       </c>
       <c r="E177" t="s">
         <v>11</v>
@@ -8486,22 +8483,22 @@
     </row>
     <row r="296" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
+        <v>343</v>
+      </c>
+      <c r="B296" t="s">
         <v>344</v>
       </c>
-      <c r="B296" t="s">
+      <c r="D296" t="s">
         <v>345</v>
       </c>
-      <c r="D296" t="s">
+      <c r="E296" t="s">
+        <v>11</v>
+      </c>
+      <c r="F296" t="s">
+        <v>344</v>
+      </c>
+      <c r="G296" t="s">
         <v>346</v>
-      </c>
-      <c r="E296" t="s">
-        <v>11</v>
-      </c>
-      <c r="F296" t="s">
-        <v>345</v>
-      </c>
-      <c r="G296" t="s">
-        <v>347</v>
       </c>
       <c r="H296" t="s">
         <v>16</v>
@@ -8512,22 +8509,22 @@
     </row>
     <row r="297" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
+        <v>343</v>
+      </c>
+      <c r="B297" t="s">
         <v>344</v>
       </c>
-      <c r="B297" t="s">
-        <v>345</v>
-      </c>
       <c r="D297" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E297" t="s">
         <v>11</v>
       </c>
       <c r="F297" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G297" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H297" t="s">
         <v>16</v>
@@ -8538,25 +8535,25 @@
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
+        <v>348</v>
+      </c>
+      <c r="B298" t="s">
         <v>349</v>
       </c>
-      <c r="B298" t="s">
+      <c r="D298" t="s">
         <v>350</v>
       </c>
-      <c r="D298" t="s">
+      <c r="E298" t="s">
+        <v>11</v>
+      </c>
+      <c r="F298" t="s">
+        <v>349</v>
+      </c>
+      <c r="G298" t="s">
+        <v>349</v>
+      </c>
+      <c r="H298" t="s">
         <v>351</v>
-      </c>
-      <c r="E298" t="s">
-        <v>11</v>
-      </c>
-      <c r="F298" t="s">
-        <v>350</v>
-      </c>
-      <c r="G298" t="s">
-        <v>350</v>
-      </c>
-      <c r="H298" t="s">
-        <v>352</v>
       </c>
       <c r="I298" t="s">
         <v>330</v>
@@ -8564,25 +8561,25 @@
     </row>
     <row r="299" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
+        <v>348</v>
+      </c>
+      <c r="B299" t="s">
         <v>349</v>
       </c>
-      <c r="B299" t="s">
-        <v>350</v>
-      </c>
       <c r="D299" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="E299" t="s">
         <v>11</v>
       </c>
       <c r="F299" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G299" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H299" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I299" t="s">
         <v>11</v>
@@ -8590,25 +8587,25 @@
     </row>
     <row r="300" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
+        <v>352</v>
+      </c>
+      <c r="B300" t="s">
+        <v>349</v>
+      </c>
+      <c r="D300" t="s">
         <v>353</v>
       </c>
-      <c r="B300" t="s">
-        <v>350</v>
-      </c>
-      <c r="D300" t="s">
-        <v>354</v>
-      </c>
       <c r="E300" t="s">
         <v>11</v>
       </c>
       <c r="F300" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G300" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H300" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I300" t="s">
         <v>330</v>
@@ -8616,25 +8613,25 @@
     </row>
     <row r="301" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B301" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D301" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="E301" t="s">
         <v>11</v>
       </c>
       <c r="F301" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G301" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H301" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="I301" t="s">
         <v>11</v>
@@ -8642,25 +8639,25 @@
     </row>
     <row r="302" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
+        <v>354</v>
+      </c>
+      <c r="B302" t="s">
         <v>355</v>
       </c>
-      <c r="B302" t="s">
+      <c r="D302" t="s">
+        <v>376</v>
+      </c>
+      <c r="E302" t="s">
+        <v>11</v>
+      </c>
+      <c r="F302" t="s">
+        <v>355</v>
+      </c>
+      <c r="G302" t="s">
         <v>356</v>
       </c>
-      <c r="D302" t="s">
-        <v>377</v>
-      </c>
-      <c r="E302" t="s">
-        <v>11</v>
-      </c>
-      <c r="F302" t="s">
-        <v>356</v>
-      </c>
-      <c r="G302" t="s">
+      <c r="H302" t="s">
         <v>357</v>
-      </c>
-      <c r="H302" t="s">
-        <v>358</v>
       </c>
       <c r="I302" t="s">
         <v>330</v>
@@ -8668,25 +8665,25 @@
     </row>
     <row r="303" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
+        <v>354</v>
+      </c>
+      <c r="B303" t="s">
         <v>355</v>
       </c>
-      <c r="B303" t="s">
+      <c r="D303" t="s">
+        <v>372</v>
+      </c>
+      <c r="E303" t="s">
+        <v>11</v>
+      </c>
+      <c r="F303" t="s">
+        <v>355</v>
+      </c>
+      <c r="G303" t="s">
         <v>356</v>
       </c>
-      <c r="D303" t="s">
-        <v>373</v>
-      </c>
-      <c r="E303" t="s">
-        <v>11</v>
-      </c>
-      <c r="F303" t="s">
-        <v>356</v>
-      </c>
-      <c r="G303" t="s">
+      <c r="H303" t="s">
         <v>357</v>
-      </c>
-      <c r="H303" t="s">
-        <v>358</v>
       </c>
       <c r="I303" t="s">
         <v>11</v>
@@ -8700,7 +8697,7 @@
         <v>123</v>
       </c>
       <c r="D304" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="E304" t="s">
         <v>11</v>
@@ -8746,22 +8743,22 @@
     </row>
     <row r="306" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
+        <v>358</v>
+      </c>
+      <c r="B306" t="s">
         <v>359</v>
       </c>
-      <c r="B306" t="s">
+      <c r="D306" t="s">
         <v>360</v>
       </c>
-      <c r="D306" t="s">
-        <v>361</v>
-      </c>
       <c r="E306" t="s">
         <v>11</v>
       </c>
       <c r="F306" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G306" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="H306" t="s">
         <v>22</v>
@@ -8772,22 +8769,22 @@
     </row>
     <row r="307" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
+        <v>358</v>
+      </c>
+      <c r="B307" t="s">
         <v>359</v>
       </c>
-      <c r="B307" t="s">
-        <v>360</v>
-      </c>
       <c r="D307" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="E307" t="s">
         <v>11</v>
       </c>
       <c r="F307" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="G307" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="H307" t="s">
         <v>22</v>
@@ -8798,13 +8795,13 @@
     </row>
     <row r="308" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
+        <v>361</v>
+      </c>
+      <c r="B308" t="s">
+        <v>127</v>
+      </c>
+      <c r="D308" t="s">
         <v>362</v>
-      </c>
-      <c r="B308" t="s">
-        <v>127</v>
-      </c>
-      <c r="D308" t="s">
-        <v>363</v>
       </c>
       <c r="E308" t="s">
         <v>11</v>
@@ -8824,13 +8821,13 @@
     </row>
     <row r="309" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="B309" t="s">
         <v>127</v>
       </c>
       <c r="D309" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="E309" t="s">
         <v>11</v>
@@ -8850,198 +8847,198 @@
     </row>
     <row r="310" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>193</v>
+        <v>364</v>
       </c>
       <c r="B310" t="s">
-        <v>127</v>
+        <v>363</v>
       </c>
       <c r="D310" t="s">
-        <v>342</v>
+        <v>365</v>
       </c>
       <c r="E310" t="s">
         <v>11</v>
       </c>
       <c r="F310" t="s">
-        <v>127</v>
+        <v>363</v>
       </c>
       <c r="G310" t="s">
-        <v>127</v>
+        <v>363</v>
       </c>
       <c r="H310" t="s">
-        <v>17</v>
+        <v>347</v>
       </c>
       <c r="I310" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
     </row>
     <row r="311" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>193</v>
+        <v>364</v>
       </c>
       <c r="B311" t="s">
-        <v>127</v>
+        <v>363</v>
       </c>
       <c r="D311" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="E311" t="s">
         <v>11</v>
       </c>
       <c r="F311" t="s">
-        <v>127</v>
+        <v>363</v>
       </c>
       <c r="G311" t="s">
-        <v>127</v>
+        <v>363</v>
       </c>
       <c r="H311" t="s">
-        <v>17</v>
-      </c>
-      <c r="I311" t="s">
-        <v>11</v>
+        <v>347</v>
       </c>
     </row>
     <row r="312" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B312" t="s">
-        <v>364</v>
+        <v>378</v>
+      </c>
+      <c r="C312" t="s">
+        <v>382</v>
       </c>
       <c r="D312" t="s">
-        <v>366</v>
-      </c>
-      <c r="E312" t="s">
-        <v>11</v>
+        <v>379</v>
       </c>
       <c r="F312" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="G312" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="H312" t="s">
-        <v>348</v>
+        <v>17</v>
       </c>
       <c r="I312" t="s">
-        <v>330</v>
+        <v>383</v>
       </c>
     </row>
     <row r="313" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="B313" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="D313" t="s">
-        <v>367</v>
-      </c>
-      <c r="E313" t="s">
-        <v>11</v>
+        <v>379</v>
       </c>
       <c r="F313" t="s">
-        <v>364</v>
+        <v>378</v>
       </c>
       <c r="G313" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="H313" t="s">
-        <v>348</v>
+        <v>17</v>
       </c>
     </row>
     <row r="314" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="B314" t="s">
-        <v>379</v>
-      </c>
-      <c r="C314" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D314" t="s">
-        <v>380</v>
+        <v>386</v>
+      </c>
+      <c r="E314" t="s">
+        <v>11</v>
       </c>
       <c r="F314" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="G314" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="H314" t="s">
-        <v>17</v>
+        <v>387</v>
       </c>
       <c r="I314" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
     </row>
     <row r="315" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
       <c r="B315" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="D315" t="s">
-        <v>380</v>
+        <v>389</v>
+      </c>
+      <c r="E315" t="s">
+        <v>11</v>
       </c>
       <c r="F315" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="G315" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="H315" t="s">
-        <v>17</v>
+        <v>387</v>
+      </c>
+      <c r="I315" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="316" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="B316" t="s">
-        <v>386</v>
+        <v>123</v>
       </c>
       <c r="D316" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="E316" t="s">
-        <v>11</v>
+        <v>392</v>
       </c>
       <c r="F316" t="s">
-        <v>386</v>
+        <v>123</v>
       </c>
       <c r="G316" t="s">
-        <v>386</v>
+        <v>123</v>
       </c>
       <c r="H316" t="s">
+        <v>27</v>
+      </c>
+      <c r="I316" t="s">
         <v>388</v>
-      </c>
-      <c r="I316" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="317" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="B317" t="s">
-        <v>386</v>
+        <v>123</v>
       </c>
       <c r="D317" t="s">
-        <v>390</v>
+        <v>419</v>
       </c>
       <c r="E317" t="s">
-        <v>11</v>
+        <v>392</v>
       </c>
       <c r="F317" t="s">
-        <v>386</v>
+        <v>123</v>
       </c>
       <c r="G317" t="s">
-        <v>386</v>
+        <v>123</v>
       </c>
       <c r="H317" t="s">
-        <v>388</v>
+        <v>27</v>
       </c>
       <c r="I317" t="s">
         <v>11</v>
@@ -9049,16 +9046,16 @@
     </row>
     <row r="318" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
+        <v>393</v>
+      </c>
+      <c r="B318" t="s">
+        <v>123</v>
+      </c>
+      <c r="D318" t="s">
         <v>391</v>
       </c>
-      <c r="B318" t="s">
-        <v>123</v>
-      </c>
-      <c r="D318" t="s">
-        <v>392</v>
-      </c>
       <c r="E318" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F318" t="s">
         <v>123</v>
@@ -9070,21 +9067,21 @@
         <v>27</v>
       </c>
       <c r="I318" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="319" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B319" t="s">
         <v>123</v>
       </c>
       <c r="D319" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E319" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F319" t="s">
         <v>123</v>
@@ -9101,16 +9098,16 @@
     </row>
     <row r="320" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B320" t="s">
         <v>123</v>
       </c>
       <c r="D320" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E320" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F320" t="s">
         <v>123</v>
@@ -9122,21 +9119,21 @@
         <v>27</v>
       </c>
       <c r="I320" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="321" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B321" t="s">
         <v>123</v>
       </c>
       <c r="D321" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E321" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F321" t="s">
         <v>123</v>
@@ -9153,16 +9150,16 @@
     </row>
     <row r="322" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B322" t="s">
         <v>123</v>
       </c>
       <c r="D322" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E322" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F322" t="s">
         <v>123</v>
@@ -9174,21 +9171,21 @@
         <v>27</v>
       </c>
       <c r="I322" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="323" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B323" t="s">
         <v>123</v>
       </c>
       <c r="D323" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E323" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F323" t="s">
         <v>123</v>
@@ -9205,16 +9202,16 @@
     </row>
     <row r="324" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B324" t="s">
         <v>123</v>
       </c>
       <c r="D324" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E324" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F324" t="s">
         <v>123</v>
@@ -9226,21 +9223,21 @@
         <v>27</v>
       </c>
       <c r="I324" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="325" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B325" t="s">
         <v>123</v>
       </c>
       <c r="D325" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E325" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="F325" t="s">
         <v>123</v>
@@ -9257,16 +9254,16 @@
     </row>
     <row r="326" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B326" t="s">
         <v>123</v>
       </c>
       <c r="D326" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E326" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F326" t="s">
         <v>123</v>
@@ -9278,21 +9275,21 @@
         <v>27</v>
       </c>
       <c r="I326" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="327" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B327" t="s">
         <v>123</v>
       </c>
       <c r="D327" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E327" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F327" t="s">
         <v>123</v>
@@ -9309,16 +9306,16 @@
     </row>
     <row r="328" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B328" t="s">
         <v>123</v>
       </c>
       <c r="D328" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E328" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F328" t="s">
         <v>123</v>
@@ -9330,21 +9327,21 @@
         <v>27</v>
       </c>
       <c r="I328" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="329" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B329" t="s">
         <v>123</v>
       </c>
       <c r="D329" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E329" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F329" t="s">
         <v>123</v>
@@ -9361,16 +9358,16 @@
     </row>
     <row r="330" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B330" t="s">
         <v>123</v>
       </c>
       <c r="D330" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E330" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F330" t="s">
         <v>123</v>
@@ -9382,21 +9379,21 @@
         <v>27</v>
       </c>
       <c r="I330" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="331" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B331" t="s">
         <v>123</v>
       </c>
       <c r="D331" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E331" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F331" t="s">
         <v>123</v>
@@ -9413,16 +9410,16 @@
     </row>
     <row r="332" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B332" t="s">
         <v>123</v>
       </c>
       <c r="D332" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E332" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F332" t="s">
         <v>123</v>
@@ -9434,21 +9431,21 @@
         <v>27</v>
       </c>
       <c r="I332" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="333" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="B333" t="s">
         <v>123</v>
       </c>
       <c r="D333" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E333" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F333" t="s">
         <v>123</v>
@@ -9465,16 +9462,16 @@
     </row>
     <row r="334" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B334" t="s">
         <v>123</v>
       </c>
       <c r="D334" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E334" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F334" t="s">
         <v>123</v>
@@ -9486,21 +9483,21 @@
         <v>27</v>
       </c>
       <c r="I334" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="335" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B335" t="s">
         <v>123</v>
       </c>
       <c r="D335" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E335" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F335" t="s">
         <v>123</v>
@@ -9517,16 +9514,16 @@
     </row>
     <row r="336" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B336" t="s">
         <v>123</v>
       </c>
       <c r="D336" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E336" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F336" t="s">
         <v>123</v>
@@ -9538,21 +9535,21 @@
         <v>27</v>
       </c>
       <c r="I336" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="337" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B337" t="s">
         <v>123</v>
       </c>
       <c r="D337" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E337" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F337" t="s">
         <v>123</v>
@@ -9569,16 +9566,16 @@
     </row>
     <row r="338" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B338" t="s">
         <v>123</v>
       </c>
       <c r="D338" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E338" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F338" t="s">
         <v>123</v>
@@ -9590,21 +9587,21 @@
         <v>27</v>
       </c>
       <c r="I338" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="339" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="B339" t="s">
         <v>123</v>
       </c>
       <c r="D339" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E339" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F339" t="s">
         <v>123</v>
@@ -9621,16 +9618,16 @@
     </row>
     <row r="340" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B340" t="s">
         <v>123</v>
       </c>
       <c r="D340" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E340" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F340" t="s">
         <v>123</v>
@@ -9642,21 +9639,21 @@
         <v>27</v>
       </c>
       <c r="I340" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="341" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B341" t="s">
         <v>123</v>
       </c>
       <c r="D341" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E341" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F341" t="s">
         <v>123</v>
@@ -9673,16 +9670,16 @@
     </row>
     <row r="342" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B342" t="s">
         <v>123</v>
       </c>
       <c r="D342" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="E342" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F342" t="s">
         <v>123</v>
@@ -9694,21 +9691,21 @@
         <v>27</v>
       </c>
       <c r="I342" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="343" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B343" t="s">
         <v>123</v>
       </c>
       <c r="D343" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="E343" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F343" t="s">
         <v>123</v>
@@ -9725,51 +9722,51 @@
     </row>
     <row r="344" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B344" t="s">
-        <v>123</v>
+        <v>421</v>
       </c>
       <c r="D344" t="s">
-        <v>392</v>
+        <v>422</v>
       </c>
       <c r="E344" t="s">
-        <v>419</v>
+        <v>11</v>
       </c>
       <c r="F344" t="s">
-        <v>123</v>
+        <v>421</v>
       </c>
       <c r="G344" t="s">
-        <v>123</v>
+        <v>421</v>
       </c>
       <c r="H344" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I344" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="345" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B345" t="s">
-        <v>123</v>
+        <v>421</v>
       </c>
       <c r="D345" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="E345" t="s">
-        <v>419</v>
+        <v>11</v>
       </c>
       <c r="F345" t="s">
-        <v>123</v>
+        <v>421</v>
       </c>
       <c r="G345" t="s">
-        <v>123</v>
+        <v>421</v>
       </c>
       <c r="H345" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="I345" t="s">
         <v>11</v>
@@ -9777,51 +9774,51 @@
     </row>
     <row r="346" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B346" t="s">
-        <v>422</v>
+        <v>9</v>
       </c>
       <c r="D346" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="E346" t="s">
         <v>11</v>
       </c>
       <c r="F346" t="s">
-        <v>422</v>
+        <v>9</v>
       </c>
       <c r="G346" t="s">
-        <v>422</v>
+        <v>9</v>
       </c>
       <c r="H346" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I346" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="347" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="B347" t="s">
-        <v>422</v>
+        <v>9</v>
       </c>
       <c r="D347" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E347" t="s">
         <v>11</v>
       </c>
       <c r="F347" t="s">
-        <v>422</v>
+        <v>9</v>
       </c>
       <c r="G347" t="s">
-        <v>422</v>
+        <v>9</v>
       </c>
       <c r="H347" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="I347" t="s">
         <v>11</v>
@@ -9829,51 +9826,51 @@
     </row>
     <row r="348" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B348" t="s">
-        <v>9</v>
+        <v>428</v>
       </c>
       <c r="D348" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="E348" t="s">
         <v>11</v>
       </c>
       <c r="F348" t="s">
-        <v>9</v>
+        <v>428</v>
       </c>
       <c r="G348" t="s">
-        <v>9</v>
+        <v>430</v>
       </c>
       <c r="H348" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I348" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="349" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B349" t="s">
-        <v>9</v>
+        <v>428</v>
       </c>
       <c r="D349" t="s">
-        <v>427</v>
+        <v>437</v>
       </c>
       <c r="E349" t="s">
         <v>11</v>
       </c>
       <c r="F349" t="s">
-        <v>9</v>
+        <v>428</v>
       </c>
       <c r="G349" t="s">
-        <v>9</v>
+        <v>430</v>
       </c>
       <c r="H349" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I349" t="s">
         <v>11</v>
@@ -9881,36 +9878,36 @@
     </row>
     <row r="350" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B350" t="s">
-        <v>429</v>
+        <v>60</v>
       </c>
       <c r="D350" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="E350" t="s">
         <v>11</v>
       </c>
       <c r="F350" t="s">
-        <v>429</v>
+        <v>60</v>
       </c>
       <c r="G350" t="s">
-        <v>431</v>
+        <v>60</v>
       </c>
       <c r="H350" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I350" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="351" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B351" t="s">
-        <v>429</v>
+        <v>60</v>
       </c>
       <c r="D351" t="s">
         <v>438</v>
@@ -9919,13 +9916,13 @@
         <v>11</v>
       </c>
       <c r="F351" t="s">
-        <v>429</v>
+        <v>60</v>
       </c>
       <c r="G351" t="s">
-        <v>431</v>
+        <v>60</v>
       </c>
       <c r="H351" t="s">
-        <v>22</v>
+        <v>57</v>
       </c>
       <c r="I351" t="s">
         <v>11</v>
@@ -9933,13 +9930,13 @@
     </row>
     <row r="352" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B352" t="s">
         <v>60</v>
       </c>
       <c r="D352" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E352" t="s">
         <v>11</v>
@@ -9954,12 +9951,12 @@
         <v>57</v>
       </c>
       <c r="I352" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="353" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B353" t="s">
         <v>60</v>
@@ -9985,13 +9982,13 @@
     </row>
     <row r="354" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B354" t="s">
         <v>60</v>
       </c>
       <c r="D354" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E354" t="s">
         <v>11</v>
@@ -10006,12 +10003,12 @@
         <v>57</v>
       </c>
       <c r="I354" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="355" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B355" t="s">
         <v>60</v>
@@ -10037,51 +10034,51 @@
     </row>
     <row r="356" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>436</v>
+        <v>445</v>
       </c>
       <c r="B356" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="D356" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="E356" t="s">
         <v>11</v>
       </c>
       <c r="F356" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="G356" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="H356" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="I356" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="357" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>436</v>
+        <v>445</v>
       </c>
       <c r="B357" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="D357" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="E357" t="s">
         <v>11</v>
       </c>
       <c r="F357" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="G357" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="H357" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="I357" t="s">
         <v>11</v>
@@ -10089,13 +10086,13 @@
     </row>
     <row r="358" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B358" t="s">
         <v>123</v>
       </c>
       <c r="D358" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E358" t="s">
         <v>11</v>
@@ -10110,12 +10107,12 @@
         <v>27</v>
       </c>
       <c r="I358" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="359" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="B359" t="s">
         <v>123</v>
@@ -10141,51 +10138,51 @@
     </row>
     <row r="360" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="B360" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D360" t="s">
-        <v>443</v>
+        <v>449</v>
       </c>
       <c r="E360" t="s">
         <v>11</v>
       </c>
       <c r="F360" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G360" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H360" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I360" t="s">
-        <v>389</v>
+        <v>311</v>
       </c>
     </row>
     <row r="361" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="B361" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="D361" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="E361" t="s">
         <v>11</v>
       </c>
       <c r="F361" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G361" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H361" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I361" t="s">
         <v>11</v>
@@ -10193,13 +10190,13 @@
     </row>
     <row r="362" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B362" t="s">
         <v>127</v>
       </c>
       <c r="D362" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="E362" t="s">
         <v>11</v>
@@ -10214,18 +10211,18 @@
         <v>17</v>
       </c>
       <c r="I362" t="s">
-        <v>311</v>
+        <v>388</v>
       </c>
     </row>
     <row r="363" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B363" t="s">
         <v>127</v>
       </c>
       <c r="D363" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E363" t="s">
         <v>11</v>
@@ -10245,13 +10242,13 @@
     </row>
     <row r="364" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>452</v>
+        <v>176</v>
       </c>
       <c r="B364" t="s">
         <v>127</v>
       </c>
       <c r="D364" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="E364" t="s">
         <v>11</v>
@@ -10266,18 +10263,18 @@
         <v>17</v>
       </c>
       <c r="I364" t="s">
-        <v>389</v>
+        <v>458</v>
       </c>
     </row>
     <row r="365" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>452</v>
+        <v>176</v>
       </c>
       <c r="B365" t="s">
         <v>127</v>
       </c>
       <c r="D365" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="E365" t="s">
         <v>11</v>
@@ -10297,13 +10294,13 @@
     </row>
     <row r="366" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>176</v>
+        <v>455</v>
       </c>
       <c r="B366" t="s">
         <v>127</v>
       </c>
       <c r="D366" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E366" t="s">
         <v>11</v>
@@ -10318,18 +10315,18 @@
         <v>17</v>
       </c>
       <c r="I366" t="s">
-        <v>459</v>
+        <v>388</v>
       </c>
     </row>
     <row r="367" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>176</v>
+        <v>455</v>
       </c>
       <c r="B367" t="s">
         <v>127</v>
       </c>
       <c r="D367" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E367" t="s">
         <v>11</v>
@@ -10349,13 +10346,13 @@
     </row>
     <row r="368" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="B368" t="s">
         <v>127</v>
       </c>
       <c r="D368" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E368" t="s">
         <v>11</v>
@@ -10370,18 +10367,18 @@
         <v>17</v>
       </c>
       <c r="I368" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="369" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
       <c r="B369" t="s">
         <v>127</v>
       </c>
       <c r="D369" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="E369" t="s">
         <v>11</v>
@@ -10401,13 +10398,13 @@
     </row>
     <row r="370" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B370" t="s">
         <v>127</v>
       </c>
       <c r="D370" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="E370" t="s">
         <v>11</v>
@@ -10422,18 +10419,18 @@
         <v>17</v>
       </c>
       <c r="I370" t="s">
-        <v>389</v>
+        <v>466</v>
       </c>
     </row>
     <row r="371" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B371" t="s">
         <v>127</v>
       </c>
       <c r="D371" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="E371" t="s">
         <v>11</v>
@@ -10453,16 +10450,16 @@
     </row>
     <row r="372" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="B372" t="s">
         <v>127</v>
       </c>
       <c r="D372" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="E372" t="s">
-        <v>11</v>
+        <v>474</v>
       </c>
       <c r="F372" t="s">
         <v>127</v>
@@ -10474,21 +10471,21 @@
         <v>17</v>
       </c>
       <c r="I372" t="s">
-        <v>467</v>
+        <v>388</v>
       </c>
     </row>
     <row r="373" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>465</v>
+        <v>475</v>
       </c>
       <c r="B373" t="s">
         <v>127</v>
       </c>
       <c r="D373" t="s">
-        <v>466</v>
+        <v>476</v>
       </c>
       <c r="E373" t="s">
-        <v>11</v>
+        <v>474</v>
       </c>
       <c r="F373" t="s">
         <v>127</v>
@@ -10505,16 +10502,16 @@
     </row>
     <row r="374" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="B374" t="s">
         <v>127</v>
       </c>
       <c r="D374" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E374" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="F374" t="s">
         <v>127</v>
@@ -10526,21 +10523,21 @@
         <v>17</v>
       </c>
       <c r="I374" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="375" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
+        <v>473</v>
+      </c>
+      <c r="B375" t="s">
+        <v>127</v>
+      </c>
+      <c r="D375" t="s">
         <v>476</v>
       </c>
-      <c r="B375" t="s">
-        <v>127</v>
-      </c>
-      <c r="D375" t="s">
-        <v>477</v>
-      </c>
       <c r="E375" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="F375" t="s">
         <v>127</v>
@@ -10557,16 +10554,16 @@
     </row>
     <row r="376" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="B376" t="s">
         <v>127</v>
       </c>
       <c r="D376" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E376" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="F376" t="s">
         <v>127</v>
@@ -10578,21 +10575,21 @@
         <v>17</v>
       </c>
       <c r="I376" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="377" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="B377" t="s">
         <v>127</v>
       </c>
       <c r="D377" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="E377" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="F377" t="s">
         <v>127</v>
@@ -10609,16 +10606,16 @@
     </row>
     <row r="378" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="B378" t="s">
         <v>127</v>
       </c>
       <c r="D378" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E378" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="F378" t="s">
         <v>127</v>
@@ -10630,21 +10627,21 @@
         <v>17</v>
       </c>
       <c r="I378" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="379" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="B379" t="s">
         <v>127</v>
       </c>
       <c r="D379" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="E379" t="s">
-        <v>471</v>
+        <v>467</v>
       </c>
       <c r="F379" t="s">
         <v>127</v>
@@ -10661,51 +10658,51 @@
     </row>
     <row r="380" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>470</v>
+        <v>487</v>
       </c>
       <c r="B380" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="D380" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
       <c r="E380" t="s">
-        <v>468</v>
+        <v>11</v>
       </c>
       <c r="F380" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="G380" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="H380" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="I380" t="s">
-        <v>389</v>
+        <v>489</v>
       </c>
     </row>
     <row r="381" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>470</v>
+        <v>487</v>
       </c>
       <c r="B381" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="D381" t="s">
-        <v>477</v>
+        <v>488</v>
       </c>
       <c r="E381" t="s">
-        <v>468</v>
+        <v>11</v>
       </c>
       <c r="F381" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="G381" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="H381" t="s">
-        <v>17</v>
+        <v>70</v>
       </c>
       <c r="I381" t="s">
         <v>11</v>
@@ -10713,13 +10710,13 @@
     </row>
     <row r="382" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="B382" t="s">
         <v>68</v>
       </c>
       <c r="D382" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="E382" t="s">
         <v>11</v>
@@ -10734,18 +10731,18 @@
         <v>70</v>
       </c>
       <c r="I382" t="s">
-        <v>490</v>
+        <v>480</v>
       </c>
     </row>
     <row r="383" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="B383" t="s">
         <v>68</v>
       </c>
       <c r="D383" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E383" t="s">
         <v>11</v>
@@ -10765,13 +10762,13 @@
     </row>
     <row r="384" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B384" t="s">
         <v>68</v>
       </c>
       <c r="D384" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="E384" t="s">
         <v>11</v>
@@ -10786,12 +10783,12 @@
         <v>70</v>
       </c>
       <c r="I384" t="s">
-        <v>481</v>
+        <v>492</v>
       </c>
     </row>
     <row r="385" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="B385" t="s">
         <v>68</v>
@@ -10817,51 +10814,51 @@
     </row>
     <row r="386" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="B386" t="s">
-        <v>68</v>
+        <v>494</v>
       </c>
       <c r="D386" t="s">
-        <v>483</v>
+        <v>495</v>
       </c>
       <c r="E386" t="s">
         <v>11</v>
       </c>
       <c r="F386" t="s">
-        <v>68</v>
+        <v>494</v>
       </c>
       <c r="G386" t="s">
-        <v>68</v>
+        <v>496</v>
       </c>
       <c r="H386" t="s">
-        <v>70</v>
+        <v>351</v>
       </c>
       <c r="I386" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
     </row>
     <row r="387" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>484</v>
+        <v>493</v>
       </c>
       <c r="B387" t="s">
-        <v>68</v>
+        <v>494</v>
       </c>
       <c r="D387" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="E387" t="s">
         <v>11</v>
       </c>
       <c r="F387" t="s">
-        <v>68</v>
+        <v>494</v>
       </c>
       <c r="G387" t="s">
-        <v>68</v>
+        <v>496</v>
       </c>
       <c r="H387" t="s">
-        <v>70</v>
+        <v>351</v>
       </c>
       <c r="I387" t="s">
         <v>11</v>
@@ -10869,51 +10866,57 @@
     </row>
     <row r="388" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>494</v>
+        <v>43</v>
       </c>
       <c r="B388" t="s">
-        <v>495</v>
+        <v>40</v>
+      </c>
+      <c r="C388" t="s">
+        <v>11</v>
       </c>
       <c r="D388" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="E388" t="s">
         <v>11</v>
       </c>
       <c r="F388" t="s">
-        <v>495</v>
+        <v>40</v>
       </c>
       <c r="G388" t="s">
-        <v>497</v>
+        <v>40</v>
       </c>
       <c r="H388" t="s">
-        <v>352</v>
+        <v>42</v>
       </c>
       <c r="I388" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
     </row>
     <row r="389" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>494</v>
+        <v>43</v>
       </c>
       <c r="B389" t="s">
-        <v>495</v>
+        <v>40</v>
+      </c>
+      <c r="C389" t="s">
+        <v>11</v>
       </c>
       <c r="D389" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="E389" t="s">
         <v>11</v>
       </c>
       <c r="F389" t="s">
-        <v>495</v>
+        <v>40</v>
       </c>
       <c r="G389" t="s">
-        <v>497</v>
+        <v>40</v>
       </c>
       <c r="H389" t="s">
-        <v>352</v>
+        <v>42</v>
       </c>
       <c r="I389" t="s">
         <v>11</v>
@@ -10921,57 +10924,57 @@
     </row>
     <row r="390" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>43</v>
+        <v>503</v>
       </c>
       <c r="B390" t="s">
-        <v>40</v>
+        <v>504</v>
       </c>
       <c r="C390" t="s">
         <v>11</v>
       </c>
       <c r="D390" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="E390" t="s">
         <v>11</v>
       </c>
       <c r="F390" t="s">
-        <v>40</v>
+        <v>504</v>
       </c>
       <c r="G390" t="s">
-        <v>40</v>
+        <v>504</v>
       </c>
       <c r="H390" t="s">
-        <v>42</v>
+        <v>506</v>
       </c>
       <c r="I390" t="s">
-        <v>503</v>
+        <v>330</v>
       </c>
     </row>
     <row r="391" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>43</v>
+        <v>503</v>
       </c>
       <c r="B391" t="s">
-        <v>40</v>
+        <v>504</v>
       </c>
       <c r="C391" t="s">
         <v>11</v>
       </c>
       <c r="D391" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
       <c r="E391" t="s">
         <v>11</v>
       </c>
       <c r="F391" t="s">
-        <v>40</v>
+        <v>504</v>
       </c>
       <c r="G391" t="s">
-        <v>40</v>
+        <v>504</v>
       </c>
       <c r="H391" t="s">
-        <v>42</v>
+        <v>506</v>
       </c>
       <c r="I391" t="s">
         <v>11</v>
@@ -10979,57 +10982,51 @@
     </row>
     <row r="392" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>504</v>
+        <v>481</v>
       </c>
       <c r="B392" t="s">
-        <v>505</v>
-      </c>
-      <c r="C392" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="D392" t="s">
-        <v>506</v>
+        <v>555</v>
       </c>
       <c r="E392" t="s">
         <v>11</v>
       </c>
       <c r="F392" t="s">
-        <v>505</v>
+        <v>68</v>
       </c>
       <c r="G392" t="s">
-        <v>505</v>
+        <v>68</v>
       </c>
       <c r="H392" t="s">
-        <v>507</v>
+        <v>70</v>
       </c>
       <c r="I392" t="s">
-        <v>330</v>
+        <v>508</v>
       </c>
     </row>
     <row r="393" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>504</v>
+        <v>481</v>
       </c>
       <c r="B393" t="s">
-        <v>505</v>
-      </c>
-      <c r="C393" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="D393" t="s">
-        <v>508</v>
+        <v>554</v>
       </c>
       <c r="E393" t="s">
         <v>11</v>
       </c>
       <c r="F393" t="s">
-        <v>505</v>
+        <v>68</v>
       </c>
       <c r="G393" t="s">
-        <v>505</v>
+        <v>68</v>
       </c>
       <c r="H393" t="s">
-        <v>507</v>
+        <v>70</v>
       </c>
       <c r="I393" t="s">
         <v>11</v>
@@ -11037,51 +11034,51 @@
     </row>
     <row r="394" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="B394" t="s">
-        <v>68</v>
+        <v>510</v>
       </c>
       <c r="D394" t="s">
-        <v>556</v>
+        <v>511</v>
       </c>
       <c r="E394" t="s">
-        <v>11</v>
+        <v>512</v>
       </c>
       <c r="F394" t="s">
-        <v>68</v>
+        <v>510</v>
       </c>
       <c r="G394" t="s">
-        <v>68</v>
+        <v>510</v>
       </c>
       <c r="H394" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="I394" t="s">
-        <v>509</v>
+        <v>552</v>
       </c>
     </row>
     <row r="395" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="B395" t="s">
-        <v>68</v>
+        <v>510</v>
       </c>
       <c r="D395" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="E395" t="s">
-        <v>11</v>
+        <v>512</v>
       </c>
       <c r="F395" t="s">
-        <v>68</v>
+        <v>510</v>
       </c>
       <c r="G395" t="s">
-        <v>68</v>
+        <v>510</v>
       </c>
       <c r="H395" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="I395" t="s">
         <v>11</v>
@@ -11089,48 +11086,48 @@
     </row>
     <row r="396" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
+        <v>513</v>
+      </c>
+      <c r="B396" t="s">
         <v>510</v>
       </c>
-      <c r="B396" t="s">
+      <c r="D396" t="s">
         <v>511</v>
       </c>
-      <c r="D396" t="s">
-        <v>512</v>
-      </c>
       <c r="E396" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F396" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="G396" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H396" t="s">
         <v>42</v>
       </c>
       <c r="I396" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="397" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
+        <v>513</v>
+      </c>
+      <c r="B397" t="s">
         <v>510</v>
       </c>
-      <c r="B397" t="s">
-        <v>511</v>
-      </c>
       <c r="D397" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="E397" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F397" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="G397" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H397" t="s">
         <v>42</v>
@@ -11141,51 +11138,57 @@
     </row>
     <row r="398" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B398" t="s">
-        <v>511</v>
+        <v>9</v>
+      </c>
+      <c r="C398" t="s">
+        <v>11</v>
       </c>
       <c r="D398" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E398" t="s">
-        <v>515</v>
+        <v>11</v>
       </c>
       <c r="F398" t="s">
-        <v>511</v>
+        <v>9</v>
       </c>
       <c r="G398" t="s">
-        <v>511</v>
+        <v>9</v>
       </c>
       <c r="H398" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="I398" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="399" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A399" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B399" t="s">
-        <v>511</v>
+        <v>9</v>
+      </c>
+      <c r="C399" t="s">
+        <v>11</v>
       </c>
       <c r="D399" t="s">
-        <v>552</v>
+        <v>540</v>
       </c>
       <c r="E399" t="s">
-        <v>515</v>
+        <v>11</v>
       </c>
       <c r="F399" t="s">
-        <v>511</v>
+        <v>9</v>
       </c>
       <c r="G399" t="s">
-        <v>511</v>
+        <v>9</v>
       </c>
       <c r="H399" t="s">
-        <v>42</v>
+        <v>12</v>
       </c>
       <c r="I399" t="s">
         <v>11</v>
@@ -11193,10 +11196,10 @@
     </row>
     <row r="400" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>516</v>
+        <v>420</v>
       </c>
       <c r="B400" t="s">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="C400" t="s">
         <v>11</v>
@@ -11208,24 +11211,24 @@
         <v>11</v>
       </c>
       <c r="F400" t="s">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="G400" t="s">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="H400" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I400" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="401" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>516</v>
+        <v>420</v>
       </c>
       <c r="B401" t="s">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="C401" t="s">
         <v>11</v>
@@ -11237,13 +11240,13 @@
         <v>11</v>
       </c>
       <c r="F401" t="s">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="G401" t="s">
-        <v>9</v>
+        <v>421</v>
       </c>
       <c r="H401" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="I401" t="s">
         <v>11</v>
@@ -11251,42 +11254,42 @@
     </row>
     <row r="402" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>421</v>
+        <v>518</v>
       </c>
       <c r="B402" t="s">
-        <v>422</v>
+        <v>349</v>
       </c>
       <c r="C402" t="s">
-        <v>11</v>
+        <v>519</v>
       </c>
       <c r="D402" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E402" t="s">
         <v>11</v>
       </c>
       <c r="F402" t="s">
-        <v>422</v>
+        <v>349</v>
       </c>
       <c r="G402" t="s">
-        <v>422</v>
+        <v>349</v>
       </c>
       <c r="H402" t="s">
-        <v>22</v>
+        <v>351</v>
       </c>
       <c r="I402" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="403" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
-        <v>421</v>
+        <v>518</v>
       </c>
       <c r="B403" t="s">
-        <v>422</v>
+        <v>349</v>
       </c>
       <c r="C403" t="s">
-        <v>11</v>
+        <v>519</v>
       </c>
       <c r="D403" t="s">
         <v>542</v>
@@ -11295,13 +11298,13 @@
         <v>11</v>
       </c>
       <c r="F403" t="s">
-        <v>422</v>
+        <v>349</v>
       </c>
       <c r="G403" t="s">
-        <v>422</v>
+        <v>349</v>
       </c>
       <c r="H403" t="s">
-        <v>22</v>
+        <v>351</v>
       </c>
       <c r="I403" t="s">
         <v>11</v>
@@ -11309,42 +11312,42 @@
     </row>
     <row r="404" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B404" t="s">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="C404" t="s">
-        <v>520</v>
+        <v>11</v>
       </c>
       <c r="D404" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E404" t="s">
         <v>11</v>
       </c>
       <c r="F404" t="s">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="G404" t="s">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="H404" t="s">
-        <v>352</v>
+        <v>17</v>
       </c>
       <c r="I404" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="405" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B405" t="s">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="C405" t="s">
-        <v>520</v>
+        <v>11</v>
       </c>
       <c r="D405" t="s">
         <v>543</v>
@@ -11353,13 +11356,13 @@
         <v>11</v>
       </c>
       <c r="F405" t="s">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="G405" t="s">
-        <v>350</v>
+        <v>522</v>
       </c>
       <c r="H405" t="s">
-        <v>352</v>
+        <v>17</v>
       </c>
       <c r="I405" t="s">
         <v>11</v>
@@ -11367,39 +11370,39 @@
     </row>
     <row r="406" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B406" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C406" t="s">
         <v>11</v>
       </c>
       <c r="D406" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E406" t="s">
         <v>11</v>
       </c>
       <c r="F406" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="G406" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="H406" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I406" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="407" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B407" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="C407" t="s">
         <v>11</v>
@@ -11411,13 +11414,13 @@
         <v>11</v>
       </c>
       <c r="F407" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="G407" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="H407" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I407" t="s">
         <v>11</v>
@@ -11425,39 +11428,39 @@
     </row>
     <row r="408" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B408" t="s">
-        <v>526</v>
+        <v>123</v>
       </c>
       <c r="C408" t="s">
         <v>11</v>
       </c>
       <c r="D408" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E408" t="s">
         <v>11</v>
       </c>
       <c r="F408" t="s">
-        <v>526</v>
+        <v>123</v>
       </c>
       <c r="G408" t="s">
-        <v>526</v>
+        <v>123</v>
       </c>
       <c r="H408" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I408" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="409" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B409" t="s">
-        <v>526</v>
+        <v>123</v>
       </c>
       <c r="C409" t="s">
         <v>11</v>
@@ -11469,13 +11472,13 @@
         <v>11</v>
       </c>
       <c r="F409" t="s">
-        <v>526</v>
+        <v>123</v>
       </c>
       <c r="G409" t="s">
-        <v>526</v>
+        <v>123</v>
       </c>
       <c r="H409" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="I409" t="s">
         <v>11</v>
@@ -11483,7 +11486,7 @@
     </row>
     <row r="410" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B410" t="s">
         <v>123</v>
@@ -11492,7 +11495,7 @@
         <v>11</v>
       </c>
       <c r="D410" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E410" t="s">
         <v>11</v>
@@ -11507,12 +11510,12 @@
         <v>27</v>
       </c>
       <c r="I410" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="411" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B411" t="s">
         <v>123</v>
@@ -11541,39 +11544,39 @@
     </row>
     <row r="412" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B412" t="s">
-        <v>123</v>
+        <v>532</v>
       </c>
       <c r="C412" t="s">
         <v>11</v>
       </c>
       <c r="D412" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="E412" t="s">
         <v>11</v>
       </c>
       <c r="F412" t="s">
-        <v>123</v>
+        <v>532</v>
       </c>
       <c r="G412" t="s">
-        <v>123</v>
+        <v>532</v>
       </c>
       <c r="H412" t="s">
-        <v>27</v>
+        <v>351</v>
       </c>
       <c r="I412" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="413" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B413" t="s">
-        <v>123</v>
+        <v>532</v>
       </c>
       <c r="C413" t="s">
         <v>11</v>
@@ -11585,13 +11588,13 @@
         <v>11</v>
       </c>
       <c r="F413" t="s">
-        <v>123</v>
+        <v>532</v>
       </c>
       <c r="G413" t="s">
-        <v>123</v>
+        <v>532</v>
       </c>
       <c r="H413" t="s">
-        <v>27</v>
+        <v>351</v>
       </c>
       <c r="I413" t="s">
         <v>11</v>
@@ -11599,42 +11602,42 @@
     </row>
     <row r="414" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B414" t="s">
-        <v>533</v>
+        <v>363</v>
       </c>
       <c r="C414" t="s">
-        <v>11</v>
+        <v>535</v>
       </c>
       <c r="D414" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="E414" t="s">
         <v>11</v>
       </c>
       <c r="F414" t="s">
-        <v>533</v>
+        <v>363</v>
       </c>
       <c r="G414" t="s">
-        <v>533</v>
+        <v>363</v>
       </c>
       <c r="H414" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="I414" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="415" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B415" t="s">
-        <v>533</v>
+        <v>363</v>
       </c>
       <c r="C415" t="s">
-        <v>11</v>
+        <v>535</v>
       </c>
       <c r="D415" t="s">
         <v>548</v>
@@ -11643,13 +11646,13 @@
         <v>11</v>
       </c>
       <c r="F415" t="s">
-        <v>533</v>
+        <v>363</v>
       </c>
       <c r="G415" t="s">
-        <v>533</v>
+        <v>363</v>
       </c>
       <c r="H415" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="I415" t="s">
         <v>11</v>
@@ -11657,42 +11660,42 @@
     </row>
     <row r="416" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B416" t="s">
-        <v>364</v>
+        <v>303</v>
       </c>
       <c r="C416" t="s">
-        <v>536</v>
+        <v>11</v>
       </c>
       <c r="D416" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E416" t="s">
         <v>11</v>
       </c>
       <c r="F416" t="s">
-        <v>364</v>
+        <v>303</v>
       </c>
       <c r="G416" t="s">
-        <v>364</v>
+        <v>303</v>
       </c>
       <c r="H416" t="s">
-        <v>348</v>
+        <v>304</v>
       </c>
       <c r="I416" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="417" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="B417" t="s">
-        <v>364</v>
+        <v>303</v>
       </c>
       <c r="C417" t="s">
-        <v>536</v>
+        <v>11</v>
       </c>
       <c r="D417" t="s">
         <v>549</v>
@@ -11701,13 +11704,13 @@
         <v>11</v>
       </c>
       <c r="F417" t="s">
-        <v>364</v>
+        <v>303</v>
       </c>
       <c r="G417" t="s">
-        <v>364</v>
+        <v>303</v>
       </c>
       <c r="H417" t="s">
-        <v>348</v>
+        <v>304</v>
       </c>
       <c r="I417" t="s">
         <v>11</v>
@@ -11715,7 +11718,7 @@
     </row>
     <row r="418" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>538</v>
+        <v>305</v>
       </c>
       <c r="B418" t="s">
         <v>303</v>
@@ -11739,12 +11742,12 @@
         <v>304</v>
       </c>
       <c r="I418" t="s">
-        <v>551</v>
+        <v>330</v>
       </c>
     </row>
     <row r="419" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>538</v>
+        <v>305</v>
       </c>
       <c r="B419" t="s">
         <v>303</v>
@@ -11753,7 +11756,7 @@
         <v>11</v>
       </c>
       <c r="D419" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="E419" t="s">
         <v>11</v>
@@ -11768,64 +11771,6 @@
         <v>304</v>
       </c>
       <c r="I419" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="420" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A420" t="s">
-        <v>305</v>
-      </c>
-      <c r="B420" t="s">
-        <v>303</v>
-      </c>
-      <c r="C420" t="s">
-        <v>11</v>
-      </c>
-      <c r="D420" t="s">
-        <v>540</v>
-      </c>
-      <c r="E420" t="s">
-        <v>11</v>
-      </c>
-      <c r="F420" t="s">
-        <v>303</v>
-      </c>
-      <c r="G420" t="s">
-        <v>303</v>
-      </c>
-      <c r="H420" t="s">
-        <v>304</v>
-      </c>
-      <c r="I420" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="421" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A421" t="s">
-        <v>305</v>
-      </c>
-      <c r="B421" t="s">
-        <v>303</v>
-      </c>
-      <c r="C421" t="s">
-        <v>11</v>
-      </c>
-      <c r="D421" t="s">
-        <v>554</v>
-      </c>
-      <c r="E421" t="s">
-        <v>11</v>
-      </c>
-      <c r="F421" t="s">
-        <v>303</v>
-      </c>
-      <c r="G421" t="s">
-        <v>303</v>
-      </c>
-      <c r="H421" t="s">
-        <v>304</v>
-      </c>
-      <c r="I421" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>